<commit_message>
Add X posting rules and update weekly flow spreadsheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FB631tAE462UfW2VKn9r6
</commit_message>
<xml_diff>
--- a/bgm/宇宙銀行_週間フロー.xlsx
+++ b/bgm/宇宙銀行_週間フロー.xlsx
@@ -15,7 +15,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nightbot設定" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="収益化" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考チャンネル10選" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="販売先・メンバーシップ" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,11 +78,6 @@
       <sz val="9"/>
       <u val="single"/>
     </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -113,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -135,55 +129,11 @@
         <color rgb="00A6A6A6"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00A6A6A6"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A6A6A6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00A6A6A6"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A6A6A6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A6A6A6"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,10 +173,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -592,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -756,21 +702,20 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>実施 18:00〜翌5:00
-（11時間・888黄金の扉）
+          <t>実施 18:00〜
+（888黄金の扉）
 ＋土曜ライブ素材づくり</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>5:00終了
-（月曜ライブ）</t>
+          <t>継続〜18:00終了</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>実施 12:00〜23:00
-（11時間・窓口の再放送）</t>
+          <t>実施 12:00〜
+（窓口の再放送）</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -785,14 +730,13 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>実施 18:00〜翌5:00
-（11時間・宇宙銀行の窓口）</t>
+          <t>実施 18:00〜
+（宇宙銀行の窓口）</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>5:00終了（土曜ライブ）
-素材準備（月曜分）
+          <t>素材準備（月曜分）
 ライブ予約</t>
         </is>
       </c>
@@ -1075,26 +1019,19 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>・ライブはすべて11時間（アーカイブが残る長さ）。月・土は18:00〜翌5:00、水は12:00〜23:00</t>
+          <t>・白蛇さんは「黄金の扉の番人」として月曜ライブの画像に時々登場させる案（未確定）</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>・白蛇さんは「黄金の扉の番人」として月曜ライブの画像に時々登場させる案（未確定）</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
           <t>・ショートとXを別の行に分けた。どちらも「窓口ワークの問いかけを1つ置いて、土曜の窓口に誘う入口」。文面は「ショート・X」シートの6週ローテーションから選ぶだけ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A15:H15"/>
@@ -1103,7 +1040,6 @@
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1117,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1511,7 +1447,7 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>窓口ワーク帳の構成を考える</t>
+          <t>窓口ワーク帳（Kindle or PDF）の構成を考える</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -1528,17 +1464,17 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>収益化</t>
+          <t>告知</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>ワーク帳をAmazonでペーパーバック＋Kindle出版</t>
+          <t>コミュニティ投稿で土曜窓口の開始を告知（紙とペンを用意）</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>「販売先・メンバーシップ」シート</t>
+          <t>初回は金曜夜に</t>
         </is>
       </c>
     </row>
@@ -1550,59 +1486,15 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>収益化</t>
+          <t>未決定</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Content IDの申し立てがある動画を確認（メンバーシップの対象外になるため）</t>
+          <t>白蛇さんの位置づけを決める</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>YouTube Studio → コンテンツ → 制限</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>告知</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>コミュニティ投稿で土曜窓口の開始を告知（紙とペンを用意）</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>初回は金曜夜に</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>未決定</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>白蛇さんの位置づけを決める</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>案：黄金の扉の番人</t>
         </is>
@@ -2461,7 +2353,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>3時間ブロックに焼き込み、ループのたびに窓口が開く設計（11時間の配信なら、0:00・3:00・6:00・9:00開始の約4回）</t>
+          <t>3時間ブロックに焼き込み、ループのたびに窓口が開く設計（24時間なら1日8回）</t>
         </is>
       </c>
     </row>
@@ -3587,372 +3479,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ワーク帳の販売先と、メンバーシップの設計</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>視聴者の中心は55〜64歳・65歳以上。「新しいアカウントを作らなくていい」「紙で書ける」を優先して選ぶ（手数料は2026年9月時点の調べ）</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>おすすめ</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>販売先</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>どんなところ</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>手数料の目安</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>チャンネル世代との相性</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="62" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>◎</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Amazon KDP
-（Kindle＋ペーパーバック）</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Amazonで電子書籍と紙の本を販売。紙の本は注文が入るたびに印刷されるので在庫なし</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>印刷代を引いた残りから、Amazonのロイヤリティ条件に沿って受け取り（Kindle出版の経験がそのまま使える）</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>◎ ほとんどの人がAmazonのアカウントを持っている。紙のワーク帳に書き込めるので窓口ワークと相性抜群</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>日本の文章・コンテンツ販売サービス。有料記事にPDFを添付して販売できる</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>クレカ決済で手取り約85%（決済手数料5%＋利用料10%）。振込ごとに270円</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>○ 名前を知っている人が多く、スマホでそのまま買える。PDFのダウンロードに慣れていない人には少し難しい</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>△</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>BOOTH</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>pixiv運営のクリエイター向けショップ。デジタル商品もグッズも販売できる</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>5.6%＋45円（2025年10月から）</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>△ 購入にpixivアカウントが必要。イラスト・同人の若い層向けの印象が強い</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>海外向け</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Gumroad</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>海外向けのデジタル商品販売サービス。英語・ドル建て</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>10%＋0.50ドル＋カード決済手数料</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>× 日本の視聴者には不向き。海外向けBGM音源の販売を始めるときの候補</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>→ まずは Amazon のペーパーバック（＋Kindle）で「宇宙銀行 窓口ワーク帳」。PDF版は note でメンバー特典や単品販売に回す</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>【メンバーシップ「窓口会員」の設計】</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>項目</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>設定内容</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>メモ</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>利用条件</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>YouTubeパートナープログラム参加中／18歳以上／子ども向け設定なし</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>音楽の申し立て（Content ID）がある動画は対象外になるので、申し立て動画は整理しておく</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>レベル数</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>最初は1つだけ（月290円前後）</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>最大6つまで作れるが、はじめはシンプルに。増やすのは会員が増えてから</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>レベル名</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>窓口会員</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>チャンネルの世界観（銀行）と合わせる</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>特典①</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>会員スタンプ（カスタム絵文字）</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>最初は4個まで。金貨・扉・宝石・「受け取ります」文字など。画像は48×48〜480×480ピクセル</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>特典②</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>継続月数で変わる会員バッジ</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n"/>
-      <c r="D17" s="20" t="n"/>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>新規＝口座開設／1か月＝普通預金／2か月＝積立預金／6か月＝定期預金／1年＝金庫会員／2年〜＝宇宙金庫会員</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>特典③</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>会員限定のコミュニティ投稿（月1回）</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>窓口ワークシートPDFや「今月の問いかけ」を配布</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>特典④</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>会員限定の窓口ライブ（月1回）</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>素材は土曜窓口の使い回しでOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>お迎えの一言</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>「宇宙銀行の窓口会員へようこそ。あなたの口座が開設されました✨」</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>入会したときの案内文</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B20:D20"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix weekly flow spreadsheet: 11h lives, Shorts 15:00, X 12:30
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FB631tAE462UfW2VKn9r6
</commit_message>
<xml_diff>
--- a/bgm/宇宙銀行_週間フロー.xlsx
+++ b/bgm/宇宙銀行_週間フロー.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週間フロー" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="やることリスト" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="視聴者の体験" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショート・X" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="窓口ワーク" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nightbot設定" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="収益化" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考チャンネル10選" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="週間フロー" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="やることリスト" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="視聴者の体験" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ショート・X" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="窓口ワーク" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Nightbot設定" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="収益化" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="参考チャンネル10選" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,7 +554,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>宇宙銀行 週間フロー（2026/9/27改訂）</t>
+          <t>宇宙銀行 週間フロー（2026/9/28改訂）</t>
         </is>
       </c>
     </row>
@@ -702,20 +702,20 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>実施 18:00〜
-（888黄金の扉）
-＋土曜ライブ素材づくり</t>
+          <t>実施 18:00〜翌5:00
+（888黄金の扉・11時間）</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>継続〜18:00終了</t>
+          <t>5:00終了
+（月曜ライブ）</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>実施 12:00〜
-（窓口の再放送）</t>
+          <t>実施 12:00〜23:00
+（月曜の再放送）</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -730,13 +730,14 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>実施 18:00〜
-（宇宙銀行の窓口）</t>
+          <t>実施 18:00〜翌5:00
+（宇宙銀行の窓口・11時間）</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>素材準備（月曜分）
+          <t>5:00終了（土曜ライブ）
+素材準備（月曜分）
 ライブ予約</t>
         </is>
       </c>
@@ -840,13 +841,13 @@
       <c r="B9" s="7" t="inlineStr">
         <is>
           <t>今週の問いかけ
-Canva制作
-→翌朝7:00予約</t>
+制作
+→翌日15:00予約</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>投稿 7:00
+          <t>投稿 15:00
 （今週の問いかけ）</t>
         </is>
       </c>
@@ -888,12 +889,12 @@
       <c r="B10" s="7" t="inlineStr">
         <is>
           <t>火曜分を予約
-（ショートと同じ問いかけ）</t>
+（12:30・ショートと同じ問いかけ）</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>投稿 7:00
+          <t>投稿 12:30
 （今週の問いかけ）</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Update weekly flow spreadsheet from latest local copy (times, Nightbot, todo status)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FB631tAE462UfW2VKn9r6
</commit_message>
<xml_diff>
--- a/bgm/宇宙銀行_週間フロー.xlsx
+++ b/bgm/宇宙銀行_週間フロー.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="週間フロー" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,16 +16,16 @@
     <sheet name="参考チャンネル10選" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -34,49 +33,75 @@
     </font>
     <font>
       <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
-      <color rgb="00595959"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <color rgb="FF595959"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
-      <b val="1"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
-      <color rgb="000563C1"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <color rgb="FF0563C1"/>
       <sz val="9"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="128"/>
+      <family val="3"/>
+      <sz val="6"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -88,22 +113,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor theme="7" tint="0.5999938962981048"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,23 +144,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="FFA6A6A6"/>
       </left>
       <right style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="FFA6A6A6"/>
       </right>
       <top style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="FFA6A6A6"/>
       </top>
       <bottom style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="FFA6A6A6"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,18 +174,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -166,16 +182,29 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -538,34 +567,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" style="12" min="1" max="1"/>
+    <col width="23" customWidth="1" style="12" min="2" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>宇宙銀行 週間フロー（2026/9/28改訂）</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="14.25" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>紫＝作業・公開がある枠／黄＝今回の変更点</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="24" customHeight="1" s="12">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>種別</t>
@@ -607,134 +630,135 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="62" customHeight="1">
+    <row r="4" ht="62.1" customHeight="1" s="12">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>3時間動画</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>制作（木曜分）</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>投稿（臨時収入）
 制作（金曜分）</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>投稿（高額当選）</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>制作（日曜分）</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>投稿（不安解消）</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
+    <row r="5" ht="62.1" customHeight="1" s="12">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>成功神殿</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>投稿（出発・今週の流れ）
 6:00</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>制作（木曜分）</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>投稿（継続・確かな自信）
 6:00</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>制作（月曜分）</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="62" customHeight="1">
+    <row r="6" ht="62.1" customHeight="1" s="12">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ライブ</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>実施 18:00〜翌5:00
-（888黄金の扉・11時間）</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
+（888黄金の扉・11時間）
+＋土曜ライブ素材づくり</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>5:00終了
 （月曜ライブ）</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>実施 12:00〜23:00
 （月曜の再放送）</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>実施 18:00〜翌5:00
 （宇宙銀行の窓口・11時間）</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>5:00終了（土曜ライブ）
 素材準備（月曜分）
@@ -742,47 +766,47 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="62" customHeight="1">
+    <row r="7" ht="62.1" customHeight="1" s="12">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>コミュニティ投稿</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>直前リマインド
 （17:30）</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>アンケート調査
 （15:30）</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>ライブ直前リマインド
 （11:30）＋成功神殿告知</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>アナリティクス分析</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>窓口リマインド（17:30）
 紙とペンを用意</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>週間まとめ＋記帳の紹介
 ＋来週予告＋成功神殿告知
@@ -790,261 +814,277 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="62" customHeight="1">
+    <row r="8" ht="62.1" customHeight="1" s="12">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Nightbot</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>共通タイマーON</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>共通タイマーON</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>共通タイマーON</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="62" customHeight="1">
+    <row r="9" ht="62.1" customHeight="1" s="12">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>ショート動画</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>今週の問いかけ
 制作
 →翌日15:00予約</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>投稿 15:00
 （今週の問いかけ）</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>窓口予告ショート制作
 →翌朝7:00予約
 （任意・同素材）</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>投稿 7:00
 （窓口予告・任意）</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="62" customHeight="1">
+    <row r="10" ht="62.1" customHeight="1" s="12">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Xのポスト</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>火曜分を予約
 （12:30・ショートと同じ問いかけ）</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>投稿 12:30
 （今週の問いかけ）</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>投稿 12:00
 （窓口リマインド）</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>投稿
 （記帳の紹介・任意）</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="62" customHeight="1">
+    <row r="11" ht="62.1" customHeight="1" s="12">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>コメント</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>5分いいね！</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="13" ht="20.1" customHeight="1" s="12">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>【変更点】</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="14" ht="20.1" customHeight="1" s="12">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>・9時間動画の行を削除（9/26から土曜はライブに変更）。月曜の「制作（前倒し）」枠は土曜ライブの素材づくりに充てる。ワーク用テロップは初回に作れば毎週使い回し可</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="15" ht="20.1" customHeight="1" s="12">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>・アンケート調査は火曜15:30</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="16" ht="20.1" customHeight="1" s="12">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>・土曜：「9時間動画告知」→「窓口リマインド（紙とペンを用意）」に変更</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>・水曜ライブは「土曜の窓口」の再放送。土曜に来られなかった人も参加でき、素材も使い回せる</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="17" ht="20.1" customHeight="1" s="12">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>・水曜ライブは当面「月曜の再放送」。10/3・10/10の窓口ライブでワークの書き込みがあれば、10/14から「窓口の再放送」に変更を検討（昼の時間帯は紙とペンのワークがしやすい）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20.1" customHeight="1" s="12">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>・日曜の週間まとめに「今週の窓口の記帳から」2〜3件の紹介を追加。チャットを読み返すのはこの時だけでOK</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="19" ht="20.1" customHeight="1" s="12">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>・Nightbotは配信中にしか動かないため、共通タイマーは常時ONのままで切り替え作業なし</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>・白蛇さんは「黄金の扉の番人」として月曜ライブの画像に時々登場させる案（未確定）</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="20" ht="20.1" customHeight="1" s="12">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>・白蛇さんは月曜ライブの画像20枚のうち2〜3枚に登場（水曜は再放送なので同じ）。「白蛇さんが現れたら、ラッキーのサイン」</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20.1" customHeight="1" s="12">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>・ショートとXを別の行に分けた。どちらも「窓口ワークの問いかけを1つ置いて、土曜の窓口に誘う入口」。文面は「ショート・X」シートの6週ローテーションから選ぶだけ</t>
         </is>
       </c>
     </row>
+    <row r="22" ht="20.1" customHeight="1" s="12">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>・ライブはすべて11時間（月・土 18:00〜翌5:00、水 12:00〜23:00）。12時間以内なのでアーカイブが残り、申し立てにも気づける</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20.1" customHeight="1" s="12">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>・ショートは火曜15:00公開（7:00より15:00のほうがよく回った実績）。Xは火曜12:30（行き先テスト中：本→チャンネル→おみくじを2週ずつ）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1055,29 +1095,29 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" style="12" min="1" max="1"/>
+    <col width="16" customWidth="1" style="12" min="2" max="2"/>
+    <col width="62" customWidth="1" style="12" min="3" max="3"/>
+    <col width="40" customWidth="1" style="12" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>やることリスト</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="14.25" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>終わったら「済」欄に ✓ を入れてください</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15.75" customHeight="1" s="12">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>済</t>
@@ -1099,411 +1139,415 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="24" customHeight="1" s="12">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>土曜窓口ライブ</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>窓口ワークのテロップを作る（案内3〜4枚×6ワーク）</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>初回だけ。以降は毎週使い回し</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="24" customHeight="1" s="12">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>土曜窓口ライブ</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>3時間ブロックにワークを焼き込んだ窓口用素材を書き出す</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>「窓口ワーク」シートの時間割どおり</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="24" customHeight="1" s="12">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>土曜窓口ライブ</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>土曜18時のライブを予約（自動スタートON）</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr"/>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+      <c r="D6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="12">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>土曜窓口ライブ</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>固定コメント「金額など個人情報は書かないでください」を用意</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr"/>
-    </row>
-    <row r="8" ht="24" customHeight="1">
+      <c r="D7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="12">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>水曜ライブ</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>水曜12時を「窓口の再放送」として予約</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>土曜と同じ素材</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>当面は月曜の再放送。10/14から窓口の再放送を検討</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" s="12">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Nightbot</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>nightbot.tv にYouTubeでログインし、Nightbotをモデレーターにする</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1" s="12">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Nightbot</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>nightbot.tv にYouTubeでログインし、Nightbotをモデレーターにする</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>共通タイマー3つを登録（チャット行数は最小値）</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>「Nightbot設定」シート①</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" s="12">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Nightbot</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>共通タイマー3つを登録（チャット行数は最小値）</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>「Nightbot設定」シート①</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>コマンド3つを登録（!madoguchi / !yokin / !uketorimasu）</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>今は「受け取ります」「888」「番号」を登録済み。窓口用は開始時に</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" s="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Nightbot</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>公開ライブ中に動くか一度確認する</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>限定公開では動かない</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1" s="12">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Nightbot</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>コマンド3つを登録（!madoguchi / !yokin / !uketorimasu）</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>「Nightbot設定」シート②</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>ショート・X</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Filmoraでショートのテンプレートを1つ作る</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>問いかけ・例・行動・締めカードの4枚</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" s="12">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Nightbot</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>公開ライブ中に動くか一度確認する</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>限定公開では動かない</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>ショート・X</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>第1週（記帳ノート）のショートとXを予約</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>「ショート・X」シート</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="12">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>収益化</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>メンバーシップの利用条件を確認し、有効にする</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-27開始「月の窓口」月額¥490</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="12">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>ショート・X</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Canvaでショートのテンプレートを1つ作る</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>問いかけ・例・行動・締めカードの4枚</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>収益化</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>会員スタンプ（カスタム絵文字）を作る</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>金貨・宇宙銀子・扉・宝石など</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" s="12">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>ショート・X</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>第1週（記帳ノート）のショートとXを予約</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>「ショート・X」シート</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>収益化</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>会員バッジの名前を設定（普通預金 → 定期預金 → 金庫会員）</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>「口座」という言葉は使わない</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="12">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>収益化</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>メンバーシップの利用条件を確認し、有効にする</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>YouTube Studio → 収益化 → メンバーシップ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>OBSにスパチャのアラート演出を入れる</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Streamlabs など</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="12">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>収益化</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>会員スタンプ（カスタム絵文字）を作る</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>金貨・宇宙銀子・扉・宝石など</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>「預金者名簿」のエンドロール用テンプレートを作る</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>週1回まとめて更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="12">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>収益化</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>窓口ワーク帳を出版する</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-27 Kindle・紙の本とも発売済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1" s="12">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>収益化</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>会員バッジの名前を設定（普通預金 → 定期預金 → 金庫会員）</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>告知</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>コミュニティ投稿で土曜窓口の開始を告知（紙とペンを用意）</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>初回は金曜夜に</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1" s="12">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>収益化</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>OBSにスパチャのアラート演出を入れる</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Streamlabs など</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>収益化</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>「預金者名簿」のエンドロール用テンプレートを作る</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>週1回まとめて更新</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>収益化</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>窓口ワーク帳（Kindle or PDF）の構成を考える</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>窓口ワーク6つ＋書き込みページ</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>告知</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>コミュニティ投稿で土曜窓口の開始を告知（紙とペンを用意）</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>初回は金曜夜に</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>未決定</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>白蛇さんの位置づけを決める</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>案：黄金の扉の番人</t>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>月曜ライブの画像に2〜3枚登場（水曜は再放送）</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1514,30 +1558,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" style="12" min="1" max="1"/>
+    <col width="40" customWidth="1" style="12" min="2" max="2"/>
+    <col width="36" customWidth="1" style="12" min="3" max="3"/>
+    <col width="32" customWidth="1" style="12" min="4" max="4"/>
+    <col width="36" customWidth="1" style="12" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>視聴者さんが窓口でやること・得られるもの</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="14.25" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>所要時間は合計15分ほど。用意するのは紙とペン、お財布、通帳かアプリだけ</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15.75" customHeight="1" s="12">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ワーク</t>
@@ -1564,177 +1608,177 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="60" customHeight="1" s="12">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>財布の窓口整理</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>レシートを全部出す／お札の向きを揃える／使わないカードを1枚抜く</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>お金を「雑に扱っていた自分」に気づく。整えた達成感がすぐ手に入る</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>財布がパンパンで、中身を把握していない</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>開くたびに気持ちいい財布。お金を丁寧に扱う感覚が戻る</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="60" customHeight="1" s="12">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>記帳ノート</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>今週受け取った小さなもの（お釣り・ポイント・おすそ分け・褒め言葉）を3つ紙に書き、財布に挟む</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>「入ってきているもの」が見えるようになる。臨時収入に気づくアンテナが立つ</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>「お金は出ていくばかり」「何も入ってこない」</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>「意外と受け取ってた」。小さな入金に日常で気づけるようになる</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="60" customHeight="1" s="12">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>今週のラッキー</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>小さなラッキーを1つ思い出して書く／当選したら最初にすることを1つ決める</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>自分は運がいい側の人間だという実感。受け取る準備ができる</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>「どうせ私には当たらない」</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>「私にもいいこと起きてる」。受け取った後の自分がイメージできる</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="60" customHeight="1" s="12">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>残高確認</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>開く前に3回息を吐いて「ありがとう」→ アプリか通帳を見る →「ここから満ちていく」と声をかける</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>数字と自分の価値を切り離せる。見ても大丈夫だった、という成功体験</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>残高を見るのが怖くて、アプリを開けない</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>週1回、落ち着いて残高を確認できる自分になる</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="60" customHeight="1" s="12">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>不安のお預け入れ</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>お金の不安を1つ紙に書き、折りたたんで封筒や引き出しにしまう</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>頭の中でぐるぐるしていた不安が「外に出る」。寝つきがよくなる</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>寝る前にお金の心配が止まらない</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>「預けたから大丈夫」と手放して眠れる</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="60" customHeight="1" s="12">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>来週の宿題</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>次にお金を払うとき、心の中で「ありがとう」と言う。翌週チャットで報告</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>支払いが「減る」から「めぐる」に変わる。毎週窓口に来る理由ができる</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>支払いのたびに、ちょっと胸がざわつく</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>支払いのたびに感謝できる。お金との関係がやわらかくなる</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="11" ht="15.75" customHeight="1" s="12">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>【通い続けたときの変化（全体のビフォーアフター）】</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
+    <row r="12" ht="15.75" customHeight="1" s="12">
+      <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>ビフォー（初めて来た日）</t>
@@ -1750,98 +1794,98 @@
           <t>3か月後</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+      <c r="E12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="12">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>お金への気持ち</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>漠然と不安。考えたくない</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>小さな入金に気づける</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>お金の話を落ち着いて考えられる</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="30" customHeight="1" s="12">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>行動</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>BGMを流すだけ</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>毎週窓口で手を動かす</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>残高確認・財布整理が習慣になる</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="30" customHeight="1" s="12">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>自分への見方</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>「私はお金に縁がない」</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>「意外と受け取ってた」</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>「私は受け取っていい人」</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="30" customHeight="1" s="12">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>チャンネルとの関係</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>たまたま流れてきた視聴者</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>土曜が楽しみな常連</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>記帳を報告し合う仲間</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="12">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>ひとことで：「BGMを流して待つ人」から「お金と向き合い、気づきを受け取れる人」へ</t>
         </is>
@@ -1849,7 +1893,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -1860,38 +1904,36 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" style="12" min="1" max="1"/>
+    <col width="18" customWidth="1" style="12" min="2" max="2"/>
+    <col width="28" customWidth="1" style="12" min="3" max="5"/>
+    <col width="60" customWidth="1" style="12" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ショート・X 運用フロー（窓口への入口）</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="14.25" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>役割：ワークを全部やってもらう場所ではなく「問いかけを1つ置いて、土曜の窓口に誘う」入口。顔出し・声なし</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+    <row r="4" ht="15.75" customHeight="1" s="12">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>【毎週のフロー】</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="15.75" customHeight="1" s="12">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>曜日</t>
@@ -1913,18 +1955,18 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="36" customHeight="1" s="12">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>① 今週のワークを選ぶ</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>下の6週ローテーション表から、今週の番号の行を開く</t>
         </is>
@@ -1935,20 +1977,20 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="36" customHeight="1" s="12">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>② ショートを作る</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Canvaのテンプレで、テロップ1〜3と締めカードの文字だけ差し替え。BGMは既存音源を15〜30秒切り出す</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Filmoraの縦長（9:16）で、テロップ1〜3と締めカードの文字だけ差し替え。背景はライブ用の画像を縦に切り抜き、BGMはIDチェック済みの音源を15〜20秒</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1957,20 +1999,20 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="36" customHeight="1" s="12">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>③ 予約する</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>ショートを火曜7:00に予約。Xの問いかけ文（下表）をコピペして火曜7:00に予約</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ショートを火曜15:00に予約（概要欄に本のURL、関連動画にライブ）。Xの問いかけ文をコピペして火曜12:30に予約</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1979,18 +2021,18 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
+    <row r="9" ht="36" customHeight="1" s="12">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>④ 窓口予告（任意）</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>同じショートの締めカードを「明日18時、窓口が開きます」に差し替えて土曜7:00に予約</t>
         </is>
@@ -2001,18 +2043,18 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1">
+    <row r="10" ht="36" customHeight="1" s="12">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>土</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>⑤ Xリマインド</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>12:00に「今夜18時、宇宙銀行の窓口が開きます。紙とペンを用意してお越しください🏦」を投稿</t>
         </is>
@@ -2023,18 +2065,18 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11" ht="36" customHeight="1" s="12">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>⑥ 記帳の紹介（任意）</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>窓口のチャットから素敵な書き込みを1つ選び、名前を伏せてXで紹介</t>
         </is>
@@ -2045,14 +2087,14 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+    <row r="13" ht="15.75" customHeight="1" s="12">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>【6週ローテーション】1週に1ワーク。6週で一周したら第1週に戻る（同じ問いかけの繰り返しでOK）</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="15.75" customHeight="1" s="12">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>週</t>
@@ -2084,8 +2126,8 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="110" customHeight="1">
-      <c r="A15" s="10" t="n">
+    <row r="15" ht="110.1" customHeight="1" s="12">
+      <c r="A15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -2093,26 +2135,26 @@
           <t>記帳ノート</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>今週、お金の形をしていない
 「入金」はありましたか？</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>お釣りの端数
 おすそ分け
 褒め言葉</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>受け取ったものを
 ひとつ書いてみてください</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>「お金は苦労しないと入ってこない」そう思っていませんか。
 今週、頑張らずに受け取ったものをひとつ思い出してみてください。お釣りの端数、おすそ分け、褒め言葉も立派な入金です。
@@ -2121,8 +2163,8 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="110" customHeight="1">
-      <c r="A16" s="10" t="n">
+    <row r="16" ht="110.1" customHeight="1" s="12">
+      <c r="A16" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -2130,25 +2172,25 @@
           <t>今週のラッキー</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>「どうせ私には当たらない」
 と思っていませんか？</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>信号がすぐ青になった
 欲しかったものが安かった</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>今週の小さなラッキーを
 ひとつ思い出してください</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>「どうせ私には当たらない」と思う前に。
 今週あった小さなラッキーをひとつ思い出してみてください。気づいた分だけ、運はあなたの味方になります。
@@ -2157,8 +2199,8 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="10" t="n">
+    <row r="17" ht="110.1" customHeight="1" s="12">
+      <c r="A17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -2166,25 +2208,25 @@
           <t>残高確認</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>残高を見るのが
 怖くありませんか？</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>それは、お金を
 大切にしてきた証です</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>開く前に3回息を吐いて
 「ありがとう」</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>残高を見るのが怖いのは、お金を大切にしてきた証です。
 開く前に3回息を吐いて「ありがとう」。見たら「ここから満ちていく」。
@@ -2194,8 +2236,8 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="110" customHeight="1">
-      <c r="A18" s="10" t="n">
+    <row r="18" ht="110.1" customHeight="1" s="12">
+      <c r="A18" s="6" t="n">
         <v>4</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -2203,25 +2245,25 @@
           <t>不安のお預け入れ</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>寝る前に
 お金の心配が止まらない夜は</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>不安をひとつ紙に書いて
 折りたたんでください</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>「宇宙銀行に
 お預けしました」</t>
         </is>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>寝る前にお金の心配が止まらない夜は、不安をひとつ紙に書いて、折りたたんでしまってください。
 「宇宙銀行にお預けしました」
@@ -2231,8 +2273,8 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="110" customHeight="1">
-      <c r="A19" s="10" t="n">
+    <row r="19" ht="110.1" customHeight="1" s="12">
+      <c r="A19" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -2240,26 +2282,26 @@
           <t>財布の窓口整理</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>お財布、パンパンに
 なっていませんか？</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>レシートを出す
 お札の向きを揃える
 カードを1枚抜く</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>5分で、お金を丁寧に
 扱う感覚が戻ります</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>財布、パンパンになっていませんか。
 レシートを出す。お札の向きを揃える。カードを1枚抜く。
@@ -2269,8 +2311,8 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="110" customHeight="1">
-      <c r="A20" s="10" t="n">
+    <row r="20" ht="110.1" customHeight="1" s="12">
+      <c r="A20" s="6" t="n">
         <v>6</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -2278,24 +2320,24 @@
           <t>ありがとう払い</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>今週の宿題です</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>次にお金を払うとき
 心の中で「ありがとう」</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>支払いは減るのではなく
 めぐっていくもの</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>今週の宿題です。
 次にお金を払うとき、心の中で「ありがとう」と言ってみてください。
@@ -2305,14 +2347,14 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="22" ht="15.75" customHeight="1" s="12">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>【締めカード（全週共通）】</t>
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="15" customHeight="1" s="12">
       <c r="A23" s="14" t="inlineStr">
         <is>
           <t>火曜ショート：「続きは土曜18時 宇宙銀行の窓口で」／土曜予告ショート：「今夜18時、窓口が開きます。紙とペンを用意してお越しください」</t>
@@ -2324,7 +2366,7 @@
     <mergeCell ref="A23:F23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -2335,30 +2377,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" style="12" min="1" max="1"/>
+    <col width="18" customWidth="1" style="12" min="2" max="2"/>
+    <col width="60" customWidth="1" style="12" min="3" max="3"/>
+    <col width="24" customWidth="1" style="12" min="4" max="4"/>
+    <col width="34" customWidth="1" style="12" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>宇宙銀行の窓口（土曜18時〜／水曜12時〜再放送）</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="14.25" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>3時間ブロックに焼き込み、ループのたびに窓口が開く設計（24時間なら1日8回）</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15.75" customHeight="1" s="12">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ブロック内の時間</t>
@@ -2385,7 +2427,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="57.95" customHeight="1" s="12">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>0:00〜</t>
@@ -2396,23 +2438,23 @@
           <t>開店の案内</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>紙とペンを用意してもらう</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="57.95" customHeight="1" s="12">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>0:10〜</t>
@@ -2423,23 +2465,23 @@
           <t>財布の窓口整理</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>レシートを出す・お札の向きを揃える・カードを1枚減らす（→5分の静かな作業画面）</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>「整えました」</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1">
+    <row r="6" ht="57.95" customHeight="1" s="12">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>0:30〜</t>
@@ -2450,23 +2492,23 @@
           <t>記帳ノート</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>今週受け取った小さなもの（お釣り・ポイント・おすそ分け・褒め言葉）を3つ書き、財布か通帳に挟む</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>受け取ったものを1つ</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>木「お金は苦労しないと入ってこない」</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="57.95" customHeight="1" s="12">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>0:40〜</t>
@@ -2477,23 +2519,23 @@
           <t>今週のラッキー</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>今週あった小さなラッキーを1つ思い出す／当選したら最初にすることを1つ書く</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>ラッキーを1つ</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>金「自分には運がない」</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1">
+    <row r="8" ht="57.95" customHeight="1" s="12">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>0:50〜</t>
@@ -2504,25 +2546,25 @@
           <t>残高確認</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>アプリか通帳を開く。①怖さを認める ②数字はあなたの価値ではない ③開く前に3回息を吐き「ありがとう」 ④見たら「ここから満ちていく」</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>「見ました」
 ※金額は書かない</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>日「お金のことを考えるのは怖い」
 土「お金はいつか尽きる」</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1">
+    <row r="9" ht="57.95" customHeight="1" s="12">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>1:10〜</t>
@@ -2533,23 +2575,23 @@
           <t>不安のお預け入れ</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>お金の不安を1つ紙に書き、折りたたんで封筒か引き出しへ。「宇宙銀行にお預けしました」</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>「預けました」</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>日「お金のことを考えるのは怖い」</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1">
+    <row r="10" ht="57.95" customHeight="1" s="12">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>1:20〜</t>
@@ -2560,23 +2602,23 @@
           <t>来週の宿題</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>次にお金を払うとき、心の中で「ありがとう」と言う。来週の窓口で報告</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>「できました」（翌週）</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1">
+    <row r="11" ht="57.95" customHeight="1" s="12">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>1:30〜3:00</t>
@@ -2587,30 +2629,30 @@
           <t>閉店・おやすみモード</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>通常のBGMループ</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>－</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="13" ht="15.75" customHeight="1" s="12">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>【曜日テーマとビリーフの対応】</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="15.75" customHeight="1" s="12">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>曜日</t>
@@ -2632,7 +2674,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="24" customHeight="1" s="12">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>木</t>
@@ -2643,18 +2685,18 @@
           <t>臨時収入</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>「お金は苦労しないと入ってこない」</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>記帳ノート</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
+    <row r="16" ht="24" customHeight="1" s="12">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>金</t>
@@ -2665,18 +2707,18 @@
           <t>高額当選</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>「自分には運がない」</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>今週のラッキー</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="24" customHeight="1" s="12">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>土</t>
@@ -2687,18 +2729,18 @@
           <t>一生お金に困らない安定</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>「お金はいつか尽きる・足りなくなる」</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>残高確認（すでにあるもの）</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
+    <row r="18" ht="24" customHeight="1" s="12">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>日</t>
@@ -2709,12 +2751,12 @@
           <t>不安解消</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>「お金のことを考えるのは怖い」</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>残高確認／不安のお預け入れ</t>
         </is>
@@ -2722,7 +2764,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -2732,50 +2774,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" style="12" min="1" max="1"/>
+    <col width="20" customWidth="1" style="12" min="2" max="2"/>
+    <col width="80" customWidth="1" style="12" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nightbot設定メモ</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+    <row r="2" ht="30" customHeight="1" s="12">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>・YouTubeでは「配信中」かつ「公開」のライブにだけ参加する（限定公開のテストでは動かない）</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="3" ht="30" customHeight="1" s="12">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>・使う前に、チャンネルでNightbotをモデレーターにする</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+    <row r="4" ht="30" customHeight="1" s="12">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>・タイマーは、指定時間が経ったあと直近5分のチャット数が設定値に達しているか確認してから投稿する。夜中は静かなので「チャット行数」は最小値に</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="6" ht="15.75" customHeight="1" s="12">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>① 共通タイマー（常時ON）</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="15.75" customHeight="1" s="12">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>名前</t>
@@ -2792,7 +2834,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="33.95" customHeight="1" s="12">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>welcome</t>
@@ -2803,13 +2845,13 @@
           <t>30〜60分</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>✨宇宙銀行へようこそ。今夜は流したまま、おやすみくださいね</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
+    <row r="9" ht="33.95" customHeight="1" s="12">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>kicho</t>
@@ -2820,13 +2862,13 @@
           <t>30〜60分</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>📖今週受け取った小さなものを、ひとつ書いてみませんか。※金額など個人情報は書かないでください</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
+    <row r="10" ht="33.95" customHeight="1" s="12">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>madoguchi</t>
@@ -2837,20 +2879,20 @@
           <t>30〜60分</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>🏦土曜18時・水曜12時は『宇宙銀行の窓口』。紙とペンを用意してお越しください</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="12" ht="15.75" customHeight="1" s="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>② コマンド（視聴者が打つと自動返信）</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="15.75" customHeight="1" s="12">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>コマンド</t>
@@ -2867,7 +2909,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="44" customHeight="1">
+    <row r="14" ht="44.1" customHeight="1" s="12">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>!madoguchi</t>
@@ -2878,13 +2920,13 @@
           <t>今日の窓口ワーク</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>🏦窓口ワーク：①財布を整える ②受け取ったものを3つ書く ③残高を見る（開く前に3回息を吐いて「ありがとう」） ④不安を紙に書いて預ける</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="44" customHeight="1">
+    <row r="15" ht="44.1" customHeight="1" s="12">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>!yokin</t>
@@ -2895,13 +2937,13 @@
           <t>不安のお預け入れ</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>🌙お金の不安をひとつ紙に書いて、折りたたんでしまってください。「宇宙銀行にお預けしました」で完了です</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1">
+    <row r="16" ht="44.1" customHeight="1" s="12">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>!uketorimasu</t>
@@ -2912,9 +2954,108 @@
           <t>受け取り</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>✨受け取りました。あなたの申込書は宇宙銀行に届いています</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>③ 今の設定（2026-09-28時点・登録済み）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1" s="12">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>コマンド／タイマー</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>返信メッセージ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44.1" customHeight="1" s="12">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>受け取ります</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>受け取り</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>✨受け取りました。あなたの申込書は宇宙銀行に届いています（名前を入れるなら先頭に $(user)さん、）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44.1" customHeight="1" s="12">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>888（8888・88888も）</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>✨888 黄金の扉が開いています。豊かさが末広がりに広がっていきますように</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44.1" customHeight="1" s="12">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>番号</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>数字おみくじ</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>「番号 8」のように書くと、各桁を足して1ケタにし、0〜9のメッセージを返す（例：✨○○さんの数字は「7」🎴 直感を信じて吉）。「8」だけだと動かない</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44.1" customHeight="1" s="12">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>タイマー：番号おみくじ</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>遊び方の案内（30分おき・2行以上）</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>🎴 数字おみくじ：チャットに「番号 8」のように好きな数字を書いてね✨（「8」だけだと動きません）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>※①の共通タイマーと②のコマンドは窓口ライブ用の予定（まだ登録していない）</t>
         </is>
       </c>
     </row>
@@ -2925,7 +3066,7 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -2936,30 +3077,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" style="12" min="1" max="1"/>
+    <col width="22" customWidth="1" style="12" min="2" max="2"/>
+    <col width="70" customWidth="1" style="12" min="3" max="3"/>
+    <col width="36" customWidth="1" style="12" min="4" max="4"/>
+    <col width="34" customWidth="1" style="12" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>収益化の仕組み（張り付かなくても回る形）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="30" customHeight="1" s="12">
       <c r="A2" s="15" t="inlineStr">
         <is>
           <t>大前提：「スパチャすると金運が上がる」とは言わない。あくまで「応援・感謝」として受け取る（開運商法に見えない／YouTubeの誤解を招くコンテンツ規約対策）</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="15.75" customHeight="1" s="12">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>優先</t>
@@ -2986,7 +3127,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="100" customHeight="1">
+    <row r="5" ht="99.95" customHeight="1" s="12">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>1</t>
@@ -2998,25 +3139,25 @@
 「窓口会員」</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>・会員スタンプ（金貨・宇宙銀子・扉・宝石のカスタム絵文字）
 ・会員限定：窓口ワークシートPDF／月1回の会員限定窓口ライブ（素材使い回し）／限定長尺版
 ・バッジ名：普通預金 → 定期預金 → 金庫会員（継続月数で変化）</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>スタンプで参加している実感、限定ワーク、続けるほど上がる「通帳ランク」</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>初回の設定とスタンプ作成のみ。以降は月1回の限定ライブ予約</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="100" customHeight="1">
+    <row r="6" ht="99.95" customHeight="1" s="12">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>2</t>
@@ -3027,24 +3168,24 @@
           <t>ワーク帳の商品化</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>・窓口ワークをまとめて Kindle本 or 印刷用ノートPDF（BOOTH／Gumroad）に
 ・概要欄・固定コメント・会員特典からリンク</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>ライブ以外の日も一人でワークできる手元のノート</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>作って置くだけ。Kindle出版のノウハウをそのまま活用</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="100" customHeight="1">
+    <row r="7" ht="99.95" customHeight="1" s="12">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>3</t>
@@ -3056,25 +3197,25 @@
 「宇宙銀行へのお預け入れ」</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>・OBSにアラート（Streamlabs等）を入れ、金貨演出＋「◯◯様のお預け入れを承りました✨」を自動表示
 ・その週の方のお名前を翌週の窓口ライブ背景に「預金者名簿」としてエンドロール表示
 ・金額帯の呼び名：「感謝の一滴」「満ちる預け入れ」など世界観に合わせる</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>画面に名前が出る喜び、名簿に刻まれる特別感</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>初回設定のみ自動。名簿は週1回まとめて作成</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="15" customHeight="1" s="12">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>※今のライブ規模（同時視聴100人前後）ではスパチャ単体はまだ小さめ。まずは毎月の土台になるメンバーシップから。</t>
@@ -3087,7 +3228,7 @@
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -3098,31 +3239,31 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" style="12" min="1" max="1"/>
+    <col width="28" customWidth="1" style="12" min="2" max="2"/>
+    <col width="20" customWidth="1" style="12" min="3" max="3"/>
+    <col width="44" customWidth="1" style="12" min="4" max="4"/>
+    <col width="40" customWidth="1" style="12" min="5" max="5"/>
+    <col width="42" customWidth="1" style="12" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="19.5" customHeight="1" s="12">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>似たことをしているチャンネル10選</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="14.25" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>「BGM×張り付かないワーク」そのものは見当たらず、要素ごとに近いものを選定。登録者数・ライブ頻度は未確認（2026/9/27調べ）</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15.75" customHeight="1" s="12">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>No.</t>
@@ -3154,11 +3295,11 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
+    <row r="4" ht="44.1" customHeight="1" s="12">
       <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>心屋仁之助【公式】</t>
         </is>
@@ -3168,27 +3309,27 @@
           <t>お金のブロック（日本）</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>「お金に恵まれない」「口ぐせを変えたい」などの公開カウンセリング</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>ビリーフを動かす言葉づかい・問いかけ方</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@kokoro-ya</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
+    <row r="5" ht="44.1" customHeight="1" s="12">
       <c r="A5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>本田晃一</t>
         </is>
@@ -3198,27 +3339,27 @@
           <t>お金のブロック（日本）</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>「世界一ゆる〜い幸せの帝王学 お金編」</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>がんばらずに受け取る語り口（木曜テーマに近い）</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=BoY3bo3DHBw</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1">
+    <row r="6" ht="44.1" customHeight="1" s="12">
       <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>本田健「Dear Ken」</t>
         </is>
@@ -3228,27 +3369,27 @@
           <t>お金のブロック（日本）</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>「お金のブロックを外すには？」などの人生相談</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>視聴者の悩みの言語化の仕方</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=yswREi_4fNc</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="44" customHeight="1">
+    <row r="7" ht="44.1" customHeight="1" s="12">
       <c r="A7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>【潜在意識・引き寄せ】探究ちゃんねる</t>
         </is>
@@ -3258,27 +3399,27 @@
           <t>潜在意識（日本）</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>潜在意識の書き換えを解説</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>潜在意識の説明の仕方（概要欄・テロップ）</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/channel/UCsDfqx5o9Z4Qac_UOGxEfLw</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1">
+    <row r="8" ht="44.1" customHeight="1" s="12">
       <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>開運＆潜在意識チャンネル</t>
         </is>
@@ -3288,27 +3429,27 @@
           <t>潜在意識（日本）</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>開運と潜在意識の掛け合わせ</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>テーマが最も近い。タイトル・サムネの比較対象に</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/channel/UCMlFv1Ou-MnfDs7w-ETX1cQ</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="44" customHeight="1">
+    <row r="9" ht="44.1" customHeight="1" s="12">
       <c r="A9" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>たかみー💰金運上昇チャンネル</t>
         </is>
@@ -3318,27 +3459,27 @@
           <t>金運実践（日本）</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>財布・金運の実践系（※Xのプロフィールから確認。YouTube側の中身は未確認）</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>財布ワークの見せ方</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>https://x.com/UP_kinun</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="44" customHeight="1">
+    <row r="10" ht="44.1" customHeight="1" s="12">
       <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Denise Duffield-Thomas</t>
         </is>
@@ -3348,27 +3489,27 @@
           <t>お金のブロック（海外）</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>money blocks（お金のブロック）解除の第一人者</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>よくあるブロック7つの整理 → 曜日別ビリーフの補強に</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/channel/UCgu5fJfr91Q0rjewdtlxUtg</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="44" customHeight="1">
+    <row r="11" ht="44.1" customHeight="1" s="12">
       <c r="A11" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Kate Northrup</t>
         </is>
@@ -3378,27 +3519,27 @@
           <t>お金と向き合う習慣（海外）</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>著書『Money: A Love Story』。定期的にお金と向き合う「お金とのデート」を提唱</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>「窓口」の考え方に最も近い。週1で通う習慣づくり</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=qFafymotfSA</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="44" customHeight="1">
+    <row r="12" ht="44.1" customHeight="1" s="12">
       <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>MONETS MONEY</t>
         </is>
@@ -3408,27 +3549,27 @@
           <t>一緒に手を動かす（海外）</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>「Budget With Me」。現金を封筒に分ける様子を毎回シリーズ配信</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>「見ながら一緒にやる」形式のシリーズ化</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=dG6oE7rJjQg</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="44" customHeight="1">
+    <row r="13" ht="44.1" customHeight="1" s="12">
       <c r="A13" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Jules Acree</t>
         </is>
@@ -3438,24 +3579,24 @@
           <t>一緒に手を動かす（海外）</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>「Real Time Journal with Me」。問いかけを出してその場で一緒に書く</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>台本を焼き込む設計に最も近い。問いかけ→書く時間の間合い</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>https://www.julesacree.com/all/journal-with-me</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="15" ht="33.95" customHeight="1" s="12">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>【ヒント】海外定番の「〜 with me」形式は、配信者が話さなくても視聴者が参加できることを示している。BGMと組み合わせたチャンネルは見当たらず、宇宙銀行の窓口は空いているポジション</t>
         </is>
@@ -3478,6 +3619,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>